<commit_message>
fix: add resistance unit warning, correct DB column header, fix solar output
- src/conductor_db.py: always treat resistance DB values as ohm/km and
  divide by 1000; added UserWarning if converted ohm/m values fall outside
  the expected range for overhead conductors
- data/conductor_data.xlsx: corrected column header from ohm/m to ohm/km
  to match the actual stored values
- conductor_ampacity.py: corrected reported solar heat gain from
  alpha*Qse*sin(theta) (W/m per diameter) to Qse (W/m²), the total solar
  and sky radiated heat intensity per IEEE 738

Co-Authored-By: Claude Sonnet 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/data/conductor_data.xlsx
+++ b/data/conductor_data.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29822"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29929"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/5e23a2a941c3b07d/notes/my_projects/conductor_ampacity/data/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="16" documentId="11_BB5F8056D34840EF615134574229E63BAD537C1D" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{970A3599-696A-4BBB-BB8C-0B3D297A3AC0}"/>
+  <xr:revisionPtr revIDLastSave="22" documentId="11_BB5F8056D34840EF615134574229E63BAD537C1D" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{A4A0B3B0-A3FB-4BE2-BF56-B1E0312E045A}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12576" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -29,12 +29,6 @@
     <t>Diameter (mm)</t>
   </si>
   <si>
-    <t>R75 (ohm/m)</t>
-  </si>
-  <si>
-    <t>R25 (ohm/m)</t>
-  </si>
-  <si>
     <t>Aluminum Weight (kg/m)</t>
   </si>
   <si>
@@ -84,6 +78,12 @@
   </si>
   <si>
     <t>Element</t>
+  </si>
+  <si>
+    <t>R75 (ohm/km)</t>
+  </si>
+  <si>
+    <t>R25 (ohm/km)</t>
   </si>
 </sst>
 </file>
@@ -517,33 +517,33 @@
         <v>1</v>
       </c>
       <c r="C1" s="3" t="s">
+        <v>19</v>
+      </c>
+      <c r="D1" s="3" t="s">
+        <v>20</v>
+      </c>
+      <c r="E1" s="3" t="s">
         <v>2</v>
       </c>
-      <c r="D1" s="3" t="s">
+      <c r="F1" s="3" t="s">
         <v>3</v>
       </c>
-      <c r="E1" s="3" t="s">
+      <c r="G1" s="3" t="s">
         <v>4</v>
       </c>
-      <c r="F1" s="3" t="s">
+      <c r="H1" s="3" t="s">
         <v>5</v>
       </c>
-      <c r="G1" s="3" t="s">
+      <c r="I1" s="3" t="s">
         <v>6</v>
       </c>
-      <c r="H1" s="3" t="s">
+      <c r="J1" s="6" t="s">
         <v>7</v>
-      </c>
-      <c r="I1" s="3" t="s">
-        <v>8</v>
-      </c>
-      <c r="J1" s="6" t="s">
-        <v>9</v>
       </c>
     </row>
     <row r="2" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A2" s="4" t="s">
-        <v>10</v>
+        <v>8</v>
       </c>
       <c r="B2" s="4">
         <v>25.15</v>
@@ -575,16 +575,16 @@
     </row>
     <row r="3" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A3" s="4" t="s">
-        <v>11</v>
+        <v>9</v>
       </c>
       <c r="B3" s="4">
-        <v>28.13</v>
+        <v>28.14</v>
       </c>
       <c r="C3" s="5">
-        <v>8.6286089238845148E-2</v>
+        <v>8.6879999999999999E-2</v>
       </c>
       <c r="D3" s="5">
-        <v>7.2344374000000003E-2</v>
+        <v>7.2830000000000006E-2</v>
       </c>
       <c r="E3" s="4">
         <v>1.1160000000000001</v>
@@ -602,12 +602,12 @@
         <v>1310</v>
       </c>
       <c r="J3" s="4">
-        <v>80</v>
+        <v>100</v>
       </c>
     </row>
     <row r="4" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A4" s="4" t="s">
-        <v>12</v>
+        <v>10</v>
       </c>
       <c r="B4" s="4">
         <v>21.78</v>
@@ -639,7 +639,7 @@
     </row>
     <row r="5" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A5" s="4" t="s">
-        <v>13</v>
+        <v>11</v>
       </c>
       <c r="B5" s="4">
         <v>28.95</v>
@@ -671,7 +671,7 @@
     </row>
     <row r="6" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A6" s="4" t="s">
-        <v>14</v>
+        <v>12</v>
       </c>
       <c r="B6" s="4">
         <v>32.83</v>
@@ -718,28 +718,28 @@
   <sheetData>
     <row r="1" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A1" s="7" t="s">
-        <v>15</v>
+        <v>13</v>
       </c>
       <c r="B1" s="8"/>
       <c r="C1" s="9"/>
     </row>
     <row r="2" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A2" s="4" t="s">
+        <v>14</v>
+      </c>
+      <c r="B2" s="4" t="s">
+        <v>15</v>
+      </c>
+      <c r="C2" s="4" t="s">
         <v>16</v>
-      </c>
-      <c r="B2" s="4" t="s">
-        <v>17</v>
-      </c>
-      <c r="C2" s="4" t="s">
-        <v>18</v>
       </c>
     </row>
     <row r="3" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A3" s="4" t="s">
-        <v>19</v>
+        <v>17</v>
       </c>
       <c r="B3" s="4" t="s">
-        <v>20</v>
+        <v>18</v>
       </c>
       <c r="C3" s="4">
         <v>3.9300000000000003E-3</v>

</xml_diff>